<commit_message>
chore: sync Nova upm-release-2026.09.28-01
</commit_message>
<xml_diff>
--- a/Assets/Samples/WechatMiniGameDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
+++ b/Assets/Samples/WechatMiniGameDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
@@ -1478,105 +1478,165 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:21">
-      <c r="B12" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>41</v>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>WeChatMiniGameVerifyLogin</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>校验微信一次性登录 code，返回 OpenID 与可选 UnionID。</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>HTTP_POST</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>GameServer</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>/v1/wx/login/verify</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:21">
-      <c r="B13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>41</v>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>WeChatMiniGameGeneratePaymentSignature</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>校验道具直购签名原文并返回 pay_sig 与 signature。</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>HTTP_POST</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>GameServer</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>/v1/wx/payment/game-item/sign</t>
+        </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:21">
-      <c r="B14" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>41</v>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>WeChatMiniGameVerifyPaymentOrders</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>批量校验 1 至 20 笔微信支付订单并返回可信状态。</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>HTTP_POST</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>GameServer</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>/v1/wx/payment/orders/verify</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:21">
-      <c r="B15" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>41</v>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>WeChatMiniGameQueryPaymentOrders</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>只读查询当前认证用户的全部服务端可见订单。</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>HTTP_POST</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>GameServer</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>/v1/wx/payment/orders/query</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:21">
-      <c r="B16" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>41</v>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>WeChatMiniGameCreateNotice</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>在微信模板授权 accept 后创建个人通知任务。</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>HTTP_POST</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>GameServer</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>/v1/wx/notice</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="2:6">
-      <c r="B17" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>41</v>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>WeChatMiniGameCheckTextContent</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>由服务端使用微信内容安全接口检查文本。</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>HTTP_POST</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>GameServer</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>/v1/wx/content/text/check</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1"/>

</xml_diff>